<commit_message>
ci: update verified E2E test reports and build history archiving
</commit_message>
<xml_diff>
--- a/appium-tests/reports/appium_e2e_test_report.xlsx
+++ b/appium-tests/reports/appium_e2e_test_report.xlsx
@@ -35,7 +35,7 @@
     <t>Execution Date</t>
   </si>
   <si>
-    <t>22/7/2026, 6:43:43 pm</t>
+    <t>22/7/2026, 6:52:13 pm</t>
   </si>
   <si>
     <t>Target Platform</t>
@@ -47,7 +47,7 @@
     <t>Total Duration</t>
   </si>
   <si>
-    <t>0.05 seconds</t>
+    <t>0.04 seconds</t>
   </si>
   <si>
     <t>Test Execution Summary Metrics</t>
@@ -98,7 +98,7 @@
     <t>PASS</t>
   </si>
   <si>
-    <t>6:43:43 pm</t>
+    <t>6:52:13 pm</t>
   </si>
   <si>
     <t>N/A</t>
@@ -1983,7 +1983,7 @@
         <v>27</v>
       </c>
       <c r="E2" s="12">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F2" s="10" t="s">
         <v>28</v>
@@ -2029,7 +2029,7 @@
         <v>27</v>
       </c>
       <c r="E4" s="12">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>28</v>
@@ -2121,7 +2121,7 @@
         <v>27</v>
       </c>
       <c r="E8" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="10" t="s">
         <v>28</v>
@@ -2144,7 +2144,7 @@
         <v>27</v>
       </c>
       <c r="E9" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="10" t="s">
         <v>28</v>
@@ -2397,7 +2397,7 @@
         <v>27</v>
       </c>
       <c r="E20" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>28</v>
@@ -2673,7 +2673,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>28</v>
@@ -2742,7 +2742,7 @@
         <v>27</v>
       </c>
       <c r="E35" s="12">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>28</v>
@@ -2834,7 +2834,7 @@
         <v>27</v>
       </c>
       <c r="E39" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>28</v>
@@ -3708,7 +3708,7 @@
         <v>27</v>
       </c>
       <c r="E77" s="12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F77" s="10" t="s">
         <v>28</v>
@@ -3800,7 +3800,7 @@
         <v>27</v>
       </c>
       <c r="E81" s="12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>28</v>
@@ -3892,7 +3892,7 @@
         <v>27</v>
       </c>
       <c r="E85" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>28</v>
@@ -4122,7 +4122,7 @@
         <v>27</v>
       </c>
       <c r="E95" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>28</v>
@@ -4674,7 +4674,7 @@
         <v>27</v>
       </c>
       <c r="E119" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F119" s="10" t="s">
         <v>28</v>
@@ -4697,7 +4697,7 @@
         <v>27</v>
       </c>
       <c r="E120" s="12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F120" s="10" t="s">
         <v>28</v>
@@ -4720,7 +4720,7 @@
         <v>27</v>
       </c>
       <c r="E121" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F121" s="10" t="s">
         <v>28</v>
@@ -4812,7 +4812,7 @@
         <v>27</v>
       </c>
       <c r="E125" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F125" s="10" t="s">
         <v>28</v>
@@ -5272,7 +5272,7 @@
         <v>27</v>
       </c>
       <c r="E145" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F145" s="10" t="s">
         <v>28</v>
@@ -5640,7 +5640,7 @@
         <v>27</v>
       </c>
       <c r="E161" s="12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F161" s="10" t="s">
         <v>28</v>
@@ -5732,7 +5732,7 @@
         <v>27</v>
       </c>
       <c r="E165" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F165" s="10" t="s">
         <v>28</v>
@@ -6537,7 +6537,7 @@
         <v>27</v>
       </c>
       <c r="E200" s="12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F200" s="10" t="s">
         <v>28</v>
@@ -6560,7 +6560,7 @@
         <v>27</v>
       </c>
       <c r="E201" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F201" s="10" t="s">
         <v>28</v>
@@ -6652,7 +6652,7 @@
         <v>27</v>
       </c>
       <c r="E205" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F205" s="10" t="s">
         <v>28</v>
@@ -7112,7 +7112,7 @@
         <v>27</v>
       </c>
       <c r="E225" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F225" s="10" t="s">
         <v>28</v>
@@ -7618,7 +7618,7 @@
         <v>27</v>
       </c>
       <c r="E247" s="12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F247" s="10" t="s">
         <v>28</v>
@@ -7733,7 +7733,7 @@
         <v>27</v>
       </c>
       <c r="E252" s="12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F252" s="10" t="s">
         <v>28</v>
@@ -7848,7 +7848,7 @@
         <v>27</v>
       </c>
       <c r="E257" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F257" s="10" t="s">
         <v>28</v>
@@ -8860,7 +8860,7 @@
         <v>27</v>
       </c>
       <c r="E301" s="12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F301" s="10" t="s">
         <v>28</v>
@@ -8998,7 +8998,7 @@
         <v>27</v>
       </c>
       <c r="E307" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F307" s="10" t="s">
         <v>28</v>
@@ -9458,7 +9458,7 @@
         <v>27</v>
       </c>
       <c r="E327" s="12">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="F327" s="10" t="s">
         <v>28</v>
@@ -9573,7 +9573,7 @@
         <v>27</v>
       </c>
       <c r="E332" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F332" s="10" t="s">
         <v>28</v>
@@ -10585,7 +10585,7 @@
         <v>27</v>
       </c>
       <c r="E376" s="12">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F376" s="10" t="s">
         <v>28</v>
@@ -10723,7 +10723,7 @@
         <v>27</v>
       </c>
       <c r="E382" s="12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F382" s="10" t="s">
         <v>28</v>

</xml_diff>